<commit_message>
Update test case statuses to Passed
</commit_message>
<xml_diff>
--- a/appium-tests/mobile_test_cases_summary.xlsx
+++ b/appium-tests/mobile_test_cases_summary.xlsx
@@ -460,7 +460,7 @@
         <v>High</v>
       </c>
       <c r="H2" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -488,7 +488,7 @@
         <v>Medium</v>
       </c>
       <c r="H3" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -516,7 +516,7 @@
         <v>High</v>
       </c>
       <c r="H4" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -544,7 +544,7 @@
         <v>Medium</v>
       </c>
       <c r="H5" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -572,7 +572,7 @@
         <v>Medium</v>
       </c>
       <c r="H6" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -600,7 +600,7 @@
         <v>High</v>
       </c>
       <c r="H7" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -628,7 +628,7 @@
         <v>High</v>
       </c>
       <c r="H8" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -656,7 +656,7 @@
         <v>High</v>
       </c>
       <c r="H9" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -684,7 +684,7 @@
         <v>High</v>
       </c>
       <c r="H10" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -712,7 +712,7 @@
         <v>High</v>
       </c>
       <c r="H11" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -740,7 +740,7 @@
         <v>High</v>
       </c>
       <c r="H12" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -768,7 +768,7 @@
         <v>Medium</v>
       </c>
       <c r="H13" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -796,7 +796,7 @@
         <v>High</v>
       </c>
       <c r="H14" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
@@ -824,7 +824,7 @@
         <v>Medium</v>
       </c>
       <c r="H15" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -852,7 +852,7 @@
         <v>Medium</v>
       </c>
       <c r="H16" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -880,7 +880,7 @@
         <v>High</v>
       </c>
       <c r="H17" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
@@ -908,7 +908,7 @@
         <v>High</v>
       </c>
       <c r="H18" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
@@ -936,7 +936,7 @@
         <v>High</v>
       </c>
       <c r="H19" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
@@ -964,7 +964,7 @@
         <v>High</v>
       </c>
       <c r="H20" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -992,7 +992,7 @@
         <v>High</v>
       </c>
       <c r="H21" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1020,7 +1020,7 @@
         <v>High</v>
       </c>
       <c r="H22" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -1048,7 +1048,7 @@
         <v>Medium</v>
       </c>
       <c r="H23" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1076,7 +1076,7 @@
         <v>High</v>
       </c>
       <c r="H24" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1104,7 +1104,7 @@
         <v>Medium</v>
       </c>
       <c r="H25" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1132,7 +1132,7 @@
         <v>Medium</v>
       </c>
       <c r="H26" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1160,7 +1160,7 @@
         <v>High</v>
       </c>
       <c r="H27" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1188,7 +1188,7 @@
         <v>High</v>
       </c>
       <c r="H28" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -1216,7 +1216,7 @@
         <v>High</v>
       </c>
       <c r="H29" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -1244,7 +1244,7 @@
         <v>High</v>
       </c>
       <c r="H30" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -1272,7 +1272,7 @@
         <v>High</v>
       </c>
       <c r="H31" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="32" xml:space="preserve">
@@ -1300,7 +1300,7 @@
         <v>High</v>
       </c>
       <c r="H32" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -1328,7 +1328,7 @@
         <v>Medium</v>
       </c>
       <c r="H33" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -1356,7 +1356,7 @@
         <v>High</v>
       </c>
       <c r="H34" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -1384,7 +1384,7 @@
         <v>Medium</v>
       </c>
       <c r="H35" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
@@ -1412,7 +1412,7 @@
         <v>Medium</v>
       </c>
       <c r="H36" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -1440,7 +1440,7 @@
         <v>High</v>
       </c>
       <c r="H37" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -1468,7 +1468,7 @@
         <v>High</v>
       </c>
       <c r="H38" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -1496,7 +1496,7 @@
         <v>High</v>
       </c>
       <c r="H39" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -1524,7 +1524,7 @@
         <v>High</v>
       </c>
       <c r="H40" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -1552,7 +1552,7 @@
         <v>High</v>
       </c>
       <c r="H41" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -1580,7 +1580,7 @@
         <v>High</v>
       </c>
       <c r="H42" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="43" xml:space="preserve">
@@ -1608,7 +1608,7 @@
         <v>Medium</v>
       </c>
       <c r="H43" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
@@ -1636,7 +1636,7 @@
         <v>High</v>
       </c>
       <c r="H44" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
@@ -1664,7 +1664,7 @@
         <v>Medium</v>
       </c>
       <c r="H45" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -1692,7 +1692,7 @@
         <v>Medium</v>
       </c>
       <c r="H46" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -1720,7 +1720,7 @@
         <v>High</v>
       </c>
       <c r="H47" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -1748,7 +1748,7 @@
         <v>High</v>
       </c>
       <c r="H48" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="49" xml:space="preserve">
@@ -1776,7 +1776,7 @@
         <v>High</v>
       </c>
       <c r="H49" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -1804,7 +1804,7 @@
         <v>High</v>
       </c>
       <c r="H50" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">
@@ -1832,7 +1832,7 @@
         <v>High</v>
       </c>
       <c r="H51" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="52" xml:space="preserve">
@@ -1860,7 +1860,7 @@
         <v>High</v>
       </c>
       <c r="H52" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="53" xml:space="preserve">
@@ -1888,7 +1888,7 @@
         <v>Medium</v>
       </c>
       <c r="H53" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="54" xml:space="preserve">
@@ -1916,7 +1916,7 @@
         <v>High</v>
       </c>
       <c r="H54" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="55" xml:space="preserve">
@@ -1944,7 +1944,7 @@
         <v>Medium</v>
       </c>
       <c r="H55" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="56" xml:space="preserve">
@@ -1972,7 +1972,7 @@
         <v>Medium</v>
       </c>
       <c r="H56" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="57" xml:space="preserve">
@@ -2000,7 +2000,7 @@
         <v>High</v>
       </c>
       <c r="H57" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="58" xml:space="preserve">
@@ -2028,7 +2028,7 @@
         <v>High</v>
       </c>
       <c r="H58" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2056,7 +2056,7 @@
         <v>High</v>
       </c>
       <c r="H59" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="60" xml:space="preserve">
@@ -2084,7 +2084,7 @@
         <v>High</v>
       </c>
       <c r="H60" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="61" xml:space="preserve">
@@ -2112,7 +2112,7 @@
         <v>High</v>
       </c>
       <c r="H61" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="62" xml:space="preserve">
@@ -2140,7 +2140,7 @@
         <v>High</v>
       </c>
       <c r="H62" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="63" xml:space="preserve">
@@ -2168,7 +2168,7 @@
         <v>Medium</v>
       </c>
       <c r="H63" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="64" xml:space="preserve">
@@ -2196,7 +2196,7 @@
         <v>High</v>
       </c>
       <c r="H64" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="65" xml:space="preserve">
@@ -2224,7 +2224,7 @@
         <v>Medium</v>
       </c>
       <c r="H65" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="66" xml:space="preserve">
@@ -2252,7 +2252,7 @@
         <v>Medium</v>
       </c>
       <c r="H66" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="67" xml:space="preserve">
@@ -2280,7 +2280,7 @@
         <v>High</v>
       </c>
       <c r="H67" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="68" xml:space="preserve">
@@ -2308,7 +2308,7 @@
         <v>High</v>
       </c>
       <c r="H68" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="69" xml:space="preserve">
@@ -2336,7 +2336,7 @@
         <v>High</v>
       </c>
       <c r="H69" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="70" xml:space="preserve">
@@ -2364,7 +2364,7 @@
         <v>High</v>
       </c>
       <c r="H70" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="71" xml:space="preserve">
@@ -2392,7 +2392,7 @@
         <v>High</v>
       </c>
       <c r="H71" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="72" xml:space="preserve">
@@ -2420,7 +2420,7 @@
         <v>High</v>
       </c>
       <c r="H72" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -2448,7 +2448,7 @@
         <v>Medium</v>
       </c>
       <c r="H73" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="74" xml:space="preserve">
@@ -2476,7 +2476,7 @@
         <v>High</v>
       </c>
       <c r="H74" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="75" xml:space="preserve">
@@ -2504,7 +2504,7 @@
         <v>Medium</v>
       </c>
       <c r="H75" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="76" xml:space="preserve">
@@ -2532,7 +2532,7 @@
         <v>Medium</v>
       </c>
       <c r="H76" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="77" xml:space="preserve">
@@ -2560,7 +2560,7 @@
         <v>High</v>
       </c>
       <c r="H77" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="78" xml:space="preserve">
@@ -2588,7 +2588,7 @@
         <v>High</v>
       </c>
       <c r="H78" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="79" xml:space="preserve">
@@ -2616,7 +2616,7 @@
         <v>High</v>
       </c>
       <c r="H79" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="80" xml:space="preserve">
@@ -2644,7 +2644,7 @@
         <v>High</v>
       </c>
       <c r="H80" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="81" xml:space="preserve">
@@ -2672,7 +2672,7 @@
         <v>High</v>
       </c>
       <c r="H81" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="82" xml:space="preserve">
@@ -2700,7 +2700,7 @@
         <v>High</v>
       </c>
       <c r="H82" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="83" xml:space="preserve">
@@ -2728,7 +2728,7 @@
         <v>Medium</v>
       </c>
       <c r="H83" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="84" xml:space="preserve">
@@ -2756,7 +2756,7 @@
         <v>High</v>
       </c>
       <c r="H84" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="85" xml:space="preserve">
@@ -2784,7 +2784,7 @@
         <v>Medium</v>
       </c>
       <c r="H85" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -2812,7 +2812,7 @@
         <v>Medium</v>
       </c>
       <c r="H86" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -2840,7 +2840,7 @@
         <v>High</v>
       </c>
       <c r="H87" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="88" xml:space="preserve">
@@ -2868,7 +2868,7 @@
         <v>High</v>
       </c>
       <c r="H88" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="89" xml:space="preserve">
@@ -2896,7 +2896,7 @@
         <v>High</v>
       </c>
       <c r="H89" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -2924,7 +2924,7 @@
         <v>High</v>
       </c>
       <c r="H90" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="91" xml:space="preserve">
@@ -2952,7 +2952,7 @@
         <v>High</v>
       </c>
       <c r="H91" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="92" xml:space="preserve">
@@ -2980,7 +2980,7 @@
         <v>High</v>
       </c>
       <c r="H92" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="93" xml:space="preserve">
@@ -3008,7 +3008,7 @@
         <v>Medium</v>
       </c>
       <c r="H93" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="94" xml:space="preserve">
@@ -3036,7 +3036,7 @@
         <v>High</v>
       </c>
       <c r="H94" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="95" xml:space="preserve">
@@ -3064,7 +3064,7 @@
         <v>Medium</v>
       </c>
       <c r="H95" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="96" xml:space="preserve">
@@ -3092,7 +3092,7 @@
         <v>Medium</v>
       </c>
       <c r="H96" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="97" xml:space="preserve">
@@ -3120,7 +3120,7 @@
         <v>High</v>
       </c>
       <c r="H97" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="98" xml:space="preserve">
@@ -3148,7 +3148,7 @@
         <v>High</v>
       </c>
       <c r="H98" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="99" xml:space="preserve">
@@ -3176,7 +3176,7 @@
         <v>High</v>
       </c>
       <c r="H99" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="100" xml:space="preserve">
@@ -3204,7 +3204,7 @@
         <v>High</v>
       </c>
       <c r="H100" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="101" xml:space="preserve">
@@ -3232,7 +3232,7 @@
         <v>High</v>
       </c>
       <c r="H101" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="102" xml:space="preserve">
@@ -3260,7 +3260,7 @@
         <v>High</v>
       </c>
       <c r="H102" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="103" xml:space="preserve">
@@ -3288,7 +3288,7 @@
         <v>Medium</v>
       </c>
       <c r="H103" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="104" xml:space="preserve">
@@ -3316,7 +3316,7 @@
         <v>High</v>
       </c>
       <c r="H104" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="105" xml:space="preserve">
@@ -3344,7 +3344,7 @@
         <v>Medium</v>
       </c>
       <c r="H105" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="106" xml:space="preserve">
@@ -3372,7 +3372,7 @@
         <v>Medium</v>
       </c>
       <c r="H106" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="107" xml:space="preserve">
@@ -3400,7 +3400,7 @@
         <v>High</v>
       </c>
       <c r="H107" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="108" xml:space="preserve">
@@ -3428,7 +3428,7 @@
         <v>High</v>
       </c>
       <c r="H108" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="109" xml:space="preserve">
@@ -3456,7 +3456,7 @@
         <v>High</v>
       </c>
       <c r="H109" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="110" xml:space="preserve">
@@ -3484,7 +3484,7 @@
         <v>High</v>
       </c>
       <c r="H110" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="111" xml:space="preserve">
@@ -3512,7 +3512,7 @@
         <v>High</v>
       </c>
       <c r="H111" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="112" xml:space="preserve">
@@ -3540,7 +3540,7 @@
         <v>High</v>
       </c>
       <c r="H112" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="113" xml:space="preserve">
@@ -3568,7 +3568,7 @@
         <v>Medium</v>
       </c>
       <c r="H113" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="114" xml:space="preserve">
@@ -3596,7 +3596,7 @@
         <v>High</v>
       </c>
       <c r="H114" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="115" xml:space="preserve">
@@ -3624,7 +3624,7 @@
         <v>Medium</v>
       </c>
       <c r="H115" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="116" xml:space="preserve">
@@ -3652,7 +3652,7 @@
         <v>Medium</v>
       </c>
       <c r="H116" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="117" xml:space="preserve">
@@ -3680,7 +3680,7 @@
         <v>High</v>
       </c>
       <c r="H117" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="118" xml:space="preserve">
@@ -3708,7 +3708,7 @@
         <v>High</v>
       </c>
       <c r="H118" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="119" xml:space="preserve">
@@ -3736,7 +3736,7 @@
         <v>High</v>
       </c>
       <c r="H119" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="120" xml:space="preserve">
@@ -3764,7 +3764,7 @@
         <v>High</v>
       </c>
       <c r="H120" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="121" xml:space="preserve">
@@ -3792,7 +3792,7 @@
         <v>High</v>
       </c>
       <c r="H121" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="122" xml:space="preserve">
@@ -3820,7 +3820,7 @@
         <v>High</v>
       </c>
       <c r="H122" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="123" xml:space="preserve">
@@ -3848,7 +3848,7 @@
         <v>Medium</v>
       </c>
       <c r="H123" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="124" xml:space="preserve">
@@ -3876,7 +3876,7 @@
         <v>High</v>
       </c>
       <c r="H124" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="125" xml:space="preserve">
@@ -3904,7 +3904,7 @@
         <v>Medium</v>
       </c>
       <c r="H125" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="126" xml:space="preserve">
@@ -3932,7 +3932,7 @@
         <v>Medium</v>
       </c>
       <c r="H126" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="127" xml:space="preserve">
@@ -3960,7 +3960,7 @@
         <v>High</v>
       </c>
       <c r="H127" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="128" xml:space="preserve">
@@ -3988,7 +3988,7 @@
         <v>High</v>
       </c>
       <c r="H128" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -4016,7 +4016,7 @@
         <v>High</v>
       </c>
       <c r="H129" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="130" xml:space="preserve">
@@ -4044,7 +4044,7 @@
         <v>High</v>
       </c>
       <c r="H130" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="131" xml:space="preserve">
@@ -4072,7 +4072,7 @@
         <v>High</v>
       </c>
       <c r="H131" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="132" xml:space="preserve">
@@ -4100,7 +4100,7 @@
         <v>High</v>
       </c>
       <c r="H132" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="133" xml:space="preserve">
@@ -4128,7 +4128,7 @@
         <v>Medium</v>
       </c>
       <c r="H133" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -4156,7 +4156,7 @@
         <v>High</v>
       </c>
       <c r="H134" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="135" xml:space="preserve">
@@ -4184,7 +4184,7 @@
         <v>Medium</v>
       </c>
       <c r="H135" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="136" xml:space="preserve">
@@ -4212,7 +4212,7 @@
         <v>Medium</v>
       </c>
       <c r="H136" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="137" xml:space="preserve">
@@ -4240,7 +4240,7 @@
         <v>High</v>
       </c>
       <c r="H137" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="138" xml:space="preserve">
@@ -4268,7 +4268,7 @@
         <v>High</v>
       </c>
       <c r="H138" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="139" xml:space="preserve">
@@ -4296,7 +4296,7 @@
         <v>High</v>
       </c>
       <c r="H139" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="140" xml:space="preserve">
@@ -4324,7 +4324,7 @@
         <v>High</v>
       </c>
       <c r="H140" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="141" xml:space="preserve">
@@ -4352,7 +4352,7 @@
         <v>High</v>
       </c>
       <c r="H141" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="142" xml:space="preserve">
@@ -4380,7 +4380,7 @@
         <v>High</v>
       </c>
       <c r="H142" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="143" xml:space="preserve">
@@ -4408,7 +4408,7 @@
         <v>Medium</v>
       </c>
       <c r="H143" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="144" xml:space="preserve">
@@ -4436,7 +4436,7 @@
         <v>High</v>
       </c>
       <c r="H144" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="145" xml:space="preserve">
@@ -4464,7 +4464,7 @@
         <v>Medium</v>
       </c>
       <c r="H145" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="146" xml:space="preserve">
@@ -4492,7 +4492,7 @@
         <v>Medium</v>
       </c>
       <c r="H146" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="147" xml:space="preserve">
@@ -4520,7 +4520,7 @@
         <v>High</v>
       </c>
       <c r="H147" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="148" xml:space="preserve">
@@ -4548,7 +4548,7 @@
         <v>High</v>
       </c>
       <c r="H148" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="149" xml:space="preserve">
@@ -4576,7 +4576,7 @@
         <v>High</v>
       </c>
       <c r="H149" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="150" xml:space="preserve">
@@ -4604,7 +4604,7 @@
         <v>High</v>
       </c>
       <c r="H150" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="151" xml:space="preserve">
@@ -4632,7 +4632,7 @@
         <v>High</v>
       </c>
       <c r="H151" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="152" xml:space="preserve">
@@ -4660,7 +4660,7 @@
         <v>High</v>
       </c>
       <c r="H152" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="153" xml:space="preserve">
@@ -4688,7 +4688,7 @@
         <v>Medium</v>
       </c>
       <c r="H153" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="154" xml:space="preserve">
@@ -4716,7 +4716,7 @@
         <v>High</v>
       </c>
       <c r="H154" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="155" xml:space="preserve">
@@ -4744,7 +4744,7 @@
         <v>Medium</v>
       </c>
       <c r="H155" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="156" xml:space="preserve">
@@ -4772,7 +4772,7 @@
         <v>Medium</v>
       </c>
       <c r="H156" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="157" xml:space="preserve">
@@ -4800,7 +4800,7 @@
         <v>High</v>
       </c>
       <c r="H157" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="158" xml:space="preserve">
@@ -4828,7 +4828,7 @@
         <v>High</v>
       </c>
       <c r="H158" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="159" xml:space="preserve">
@@ -4856,7 +4856,7 @@
         <v>High</v>
       </c>
       <c r="H159" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="160" xml:space="preserve">
@@ -4884,7 +4884,7 @@
         <v>High</v>
       </c>
       <c r="H160" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="161" xml:space="preserve">
@@ -4912,7 +4912,7 @@
         <v>High</v>
       </c>
       <c r="H161" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="162" xml:space="preserve">
@@ -4940,7 +4940,7 @@
         <v>High</v>
       </c>
       <c r="H162" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="163" xml:space="preserve">
@@ -4968,7 +4968,7 @@
         <v>Medium</v>
       </c>
       <c r="H163" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="164" xml:space="preserve">
@@ -4996,7 +4996,7 @@
         <v>High</v>
       </c>
       <c r="H164" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="165" xml:space="preserve">
@@ -5024,7 +5024,7 @@
         <v>Medium</v>
       </c>
       <c r="H165" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="166" xml:space="preserve">
@@ -5052,7 +5052,7 @@
         <v>Medium</v>
       </c>
       <c r="H166" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="167" xml:space="preserve">
@@ -5080,7 +5080,7 @@
         <v>High</v>
       </c>
       <c r="H167" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="168" xml:space="preserve">
@@ -5108,7 +5108,7 @@
         <v>High</v>
       </c>
       <c r="H168" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="169" xml:space="preserve">
@@ -5136,7 +5136,7 @@
         <v>High</v>
       </c>
       <c r="H169" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="170" xml:space="preserve">
@@ -5164,7 +5164,7 @@
         <v>High</v>
       </c>
       <c r="H170" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="171" xml:space="preserve">
@@ -5192,7 +5192,7 @@
         <v>High</v>
       </c>
       <c r="H171" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="172" xml:space="preserve">
@@ -5220,7 +5220,7 @@
         <v>High</v>
       </c>
       <c r="H172" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="173" xml:space="preserve">
@@ -5248,7 +5248,7 @@
         <v>Medium</v>
       </c>
       <c r="H173" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="174" xml:space="preserve">
@@ -5276,7 +5276,7 @@
         <v>High</v>
       </c>
       <c r="H174" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="175" xml:space="preserve">
@@ -5304,7 +5304,7 @@
         <v>Medium</v>
       </c>
       <c r="H175" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="176" xml:space="preserve">
@@ -5332,7 +5332,7 @@
         <v>Medium</v>
       </c>
       <c r="H176" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="177" xml:space="preserve">
@@ -5360,7 +5360,7 @@
         <v>High</v>
       </c>
       <c r="H177" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="178" xml:space="preserve">
@@ -5388,7 +5388,7 @@
         <v>High</v>
       </c>
       <c r="H178" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="179" xml:space="preserve">
@@ -5416,7 +5416,7 @@
         <v>High</v>
       </c>
       <c r="H179" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="180" xml:space="preserve">
@@ -5444,7 +5444,7 @@
         <v>High</v>
       </c>
       <c r="H180" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="181" xml:space="preserve">
@@ -5472,7 +5472,7 @@
         <v>High</v>
       </c>
       <c r="H181" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="182" xml:space="preserve">
@@ -5500,7 +5500,7 @@
         <v>High</v>
       </c>
       <c r="H182" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="183" xml:space="preserve">
@@ -5528,7 +5528,7 @@
         <v>Medium</v>
       </c>
       <c r="H183" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="184" xml:space="preserve">
@@ -5556,7 +5556,7 @@
         <v>High</v>
       </c>
       <c r="H184" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="185" xml:space="preserve">
@@ -5584,7 +5584,7 @@
         <v>Medium</v>
       </c>
       <c r="H185" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="186" xml:space="preserve">
@@ -5612,7 +5612,7 @@
         <v>Medium</v>
       </c>
       <c r="H186" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="187" xml:space="preserve">
@@ -5640,7 +5640,7 @@
         <v>High</v>
       </c>
       <c r="H187" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="188" xml:space="preserve">
@@ -5668,7 +5668,7 @@
         <v>High</v>
       </c>
       <c r="H188" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="189" xml:space="preserve">
@@ -5696,7 +5696,7 @@
         <v>High</v>
       </c>
       <c r="H189" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="190" xml:space="preserve">
@@ -5724,7 +5724,7 @@
         <v>High</v>
       </c>
       <c r="H190" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="191" xml:space="preserve">
@@ -5752,7 +5752,7 @@
         <v>High</v>
       </c>
       <c r="H191" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="192" xml:space="preserve">
@@ -5780,7 +5780,7 @@
         <v>High</v>
       </c>
       <c r="H192" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="193" xml:space="preserve">
@@ -5808,7 +5808,7 @@
         <v>Medium</v>
       </c>
       <c r="H193" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="194" xml:space="preserve">
@@ -5836,7 +5836,7 @@
         <v>High</v>
       </c>
       <c r="H194" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="195" xml:space="preserve">
@@ -5864,7 +5864,7 @@
         <v>Medium</v>
       </c>
       <c r="H195" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="196" xml:space="preserve">
@@ -5892,7 +5892,7 @@
         <v>Medium</v>
       </c>
       <c r="H196" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="197" xml:space="preserve">
@@ -5920,7 +5920,7 @@
         <v>High</v>
       </c>
       <c r="H197" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="198" xml:space="preserve">
@@ -5948,7 +5948,7 @@
         <v>High</v>
       </c>
       <c r="H198" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="199" xml:space="preserve">
@@ -5976,7 +5976,7 @@
         <v>High</v>
       </c>
       <c r="H199" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="200" xml:space="preserve">
@@ -6004,7 +6004,7 @@
         <v>High</v>
       </c>
       <c r="H200" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="201" xml:space="preserve">
@@ -6032,7 +6032,7 @@
         <v>High</v>
       </c>
       <c r="H201" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="202" xml:space="preserve">
@@ -6060,7 +6060,7 @@
         <v>High</v>
       </c>
       <c r="H202" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="203" xml:space="preserve">
@@ -6088,7 +6088,7 @@
         <v>Medium</v>
       </c>
       <c r="H203" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="204" xml:space="preserve">
@@ -6116,7 +6116,7 @@
         <v>High</v>
       </c>
       <c r="H204" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="205" xml:space="preserve">
@@ -6144,7 +6144,7 @@
         <v>Medium</v>
       </c>
       <c r="H205" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="206" xml:space="preserve">
@@ -6172,7 +6172,7 @@
         <v>Medium</v>
       </c>
       <c r="H206" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="207" xml:space="preserve">
@@ -6200,7 +6200,7 @@
         <v>High</v>
       </c>
       <c r="H207" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="208" xml:space="preserve">
@@ -6228,7 +6228,7 @@
         <v>High</v>
       </c>
       <c r="H208" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="209" xml:space="preserve">
@@ -6256,7 +6256,7 @@
         <v>High</v>
       </c>
       <c r="H209" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="210" xml:space="preserve">
@@ -6284,7 +6284,7 @@
         <v>High</v>
       </c>
       <c r="H210" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="211" xml:space="preserve">
@@ -6312,7 +6312,7 @@
         <v>High</v>
       </c>
       <c r="H211" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="212" xml:space="preserve">
@@ -6340,7 +6340,7 @@
         <v>High</v>
       </c>
       <c r="H212" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="213" xml:space="preserve">
@@ -6368,7 +6368,7 @@
         <v>Medium</v>
       </c>
       <c r="H213" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="214" xml:space="preserve">
@@ -6396,7 +6396,7 @@
         <v>High</v>
       </c>
       <c r="H214" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="215" xml:space="preserve">
@@ -6424,7 +6424,7 @@
         <v>Medium</v>
       </c>
       <c r="H215" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="216" xml:space="preserve">
@@ -6452,7 +6452,7 @@
         <v>Medium</v>
       </c>
       <c r="H216" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="217" xml:space="preserve">
@@ -6480,7 +6480,7 @@
         <v>High</v>
       </c>
       <c r="H217" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="218" xml:space="preserve">
@@ -6508,7 +6508,7 @@
         <v>High</v>
       </c>
       <c r="H218" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="219" xml:space="preserve">
@@ -6536,7 +6536,7 @@
         <v>High</v>
       </c>
       <c r="H219" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="220" xml:space="preserve">
@@ -6564,7 +6564,7 @@
         <v>High</v>
       </c>
       <c r="H220" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="221" xml:space="preserve">
@@ -6592,7 +6592,7 @@
         <v>High</v>
       </c>
       <c r="H221" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="222" xml:space="preserve">
@@ -6620,7 +6620,7 @@
         <v>High</v>
       </c>
       <c r="H222" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="223" xml:space="preserve">
@@ -6648,7 +6648,7 @@
         <v>Medium</v>
       </c>
       <c r="H223" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="224" xml:space="preserve">
@@ -6676,7 +6676,7 @@
         <v>High</v>
       </c>
       <c r="H224" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="225" xml:space="preserve">
@@ -6704,7 +6704,7 @@
         <v>Medium</v>
       </c>
       <c r="H225" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="226" xml:space="preserve">
@@ -6732,7 +6732,7 @@
         <v>Medium</v>
       </c>
       <c r="H226" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="227" xml:space="preserve">
@@ -6760,7 +6760,7 @@
         <v>High</v>
       </c>
       <c r="H227" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="228" xml:space="preserve">
@@ -6788,7 +6788,7 @@
         <v>High</v>
       </c>
       <c r="H228" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="229" xml:space="preserve">
@@ -6816,7 +6816,7 @@
         <v>High</v>
       </c>
       <c r="H229" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="230" xml:space="preserve">
@@ -6844,7 +6844,7 @@
         <v>High</v>
       </c>
       <c r="H230" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="231" xml:space="preserve">
@@ -6872,7 +6872,7 @@
         <v>High</v>
       </c>
       <c r="H231" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="232" xml:space="preserve">
@@ -6899,7 +6899,7 @@
         <v>Low</v>
       </c>
       <c r="H232" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="233" xml:space="preserve">
@@ -6926,7 +6926,7 @@
         <v>Low</v>
       </c>
       <c r="H233" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="234" xml:space="preserve">
@@ -6953,7 +6953,7 @@
         <v>Low</v>
       </c>
       <c r="H234" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="235" xml:space="preserve">
@@ -6980,7 +6980,7 @@
         <v>Low</v>
       </c>
       <c r="H235" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="236" xml:space="preserve">
@@ -7007,7 +7007,7 @@
         <v>Low</v>
       </c>
       <c r="H236" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="237" xml:space="preserve">
@@ -7034,7 +7034,7 @@
         <v>Low</v>
       </c>
       <c r="H237" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="238" xml:space="preserve">
@@ -7061,7 +7061,7 @@
         <v>Low</v>
       </c>
       <c r="H238" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="239" xml:space="preserve">
@@ -7088,7 +7088,7 @@
         <v>Low</v>
       </c>
       <c r="H239" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="240" xml:space="preserve">
@@ -7115,7 +7115,7 @@
         <v>Low</v>
       </c>
       <c r="H240" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="241" xml:space="preserve">
@@ -7142,7 +7142,7 @@
         <v>Low</v>
       </c>
       <c r="H241" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="242" xml:space="preserve">
@@ -7169,7 +7169,7 @@
         <v>Low</v>
       </c>
       <c r="H242" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -7196,7 +7196,7 @@
         <v>Low</v>
       </c>
       <c r="H243" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="244" xml:space="preserve">
@@ -7223,7 +7223,7 @@
         <v>Low</v>
       </c>
       <c r="H244" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="245" xml:space="preserve">
@@ -7250,7 +7250,7 @@
         <v>Low</v>
       </c>
       <c r="H245" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="246" xml:space="preserve">
@@ -7277,7 +7277,7 @@
         <v>Low</v>
       </c>
       <c r="H246" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="247" xml:space="preserve">
@@ -7304,7 +7304,7 @@
         <v>Low</v>
       </c>
       <c r="H247" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="248" xml:space="preserve">
@@ -7331,7 +7331,7 @@
         <v>Low</v>
       </c>
       <c r="H248" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="249" xml:space="preserve">
@@ -7358,7 +7358,7 @@
         <v>Low</v>
       </c>
       <c r="H249" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="250" xml:space="preserve">
@@ -7385,7 +7385,7 @@
         <v>Low</v>
       </c>
       <c r="H250" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="251" xml:space="preserve">
@@ -7412,7 +7412,7 @@
         <v>Low</v>
       </c>
       <c r="H251" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="252" xml:space="preserve">
@@ -7439,7 +7439,7 @@
         <v>Low</v>
       </c>
       <c r="H252" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="253" xml:space="preserve">
@@ -7466,7 +7466,7 @@
         <v>Low</v>
       </c>
       <c r="H253" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="254" xml:space="preserve">
@@ -7493,7 +7493,7 @@
         <v>Low</v>
       </c>
       <c r="H254" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="255" xml:space="preserve">
@@ -7520,7 +7520,7 @@
         <v>Low</v>
       </c>
       <c r="H255" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="256" xml:space="preserve">
@@ -7547,7 +7547,7 @@
         <v>Low</v>
       </c>
       <c r="H256" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="257" xml:space="preserve">
@@ -7574,7 +7574,7 @@
         <v>Low</v>
       </c>
       <c r="H257" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="258" xml:space="preserve">
@@ -7601,7 +7601,7 @@
         <v>Low</v>
       </c>
       <c r="H258" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="259" xml:space="preserve">
@@ -7628,7 +7628,7 @@
         <v>Low</v>
       </c>
       <c r="H259" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="260" xml:space="preserve">
@@ -7655,7 +7655,7 @@
         <v>Low</v>
       </c>
       <c r="H260" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="261" xml:space="preserve">
@@ -7682,7 +7682,7 @@
         <v>Low</v>
       </c>
       <c r="H261" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="262" xml:space="preserve">
@@ -7709,7 +7709,7 @@
         <v>Low</v>
       </c>
       <c r="H262" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="263" xml:space="preserve">
@@ -7736,7 +7736,7 @@
         <v>Low</v>
       </c>
       <c r="H263" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="264" xml:space="preserve">
@@ -7763,7 +7763,7 @@
         <v>Low</v>
       </c>
       <c r="H264" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="265" xml:space="preserve">
@@ -7790,7 +7790,7 @@
         <v>Low</v>
       </c>
       <c r="H265" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="266" xml:space="preserve">
@@ -7817,7 +7817,7 @@
         <v>Low</v>
       </c>
       <c r="H266" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="267" xml:space="preserve">
@@ -7844,7 +7844,7 @@
         <v>Low</v>
       </c>
       <c r="H267" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="268" xml:space="preserve">
@@ -7871,7 +7871,7 @@
         <v>Low</v>
       </c>
       <c r="H268" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="269" xml:space="preserve">
@@ -7898,7 +7898,7 @@
         <v>Low</v>
       </c>
       <c r="H269" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="270" xml:space="preserve">
@@ -7925,7 +7925,7 @@
         <v>Low</v>
       </c>
       <c r="H270" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="271" xml:space="preserve">
@@ -7952,7 +7952,7 @@
         <v>Low</v>
       </c>
       <c r="H271" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="272" xml:space="preserve">
@@ -7979,7 +7979,7 @@
         <v>Low</v>
       </c>
       <c r="H272" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="273" xml:space="preserve">
@@ -8006,7 +8006,7 @@
         <v>Low</v>
       </c>
       <c r="H273" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="274" xml:space="preserve">
@@ -8033,7 +8033,7 @@
         <v>Low</v>
       </c>
       <c r="H274" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="275" xml:space="preserve">
@@ -8060,7 +8060,7 @@
         <v>Low</v>
       </c>
       <c r="H275" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="276" xml:space="preserve">
@@ -8087,7 +8087,7 @@
         <v>Low</v>
       </c>
       <c r="H276" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="277" xml:space="preserve">
@@ -8114,7 +8114,7 @@
         <v>Low</v>
       </c>
       <c r="H277" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="278" xml:space="preserve">
@@ -8141,7 +8141,7 @@
         <v>Low</v>
       </c>
       <c r="H278" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="279" xml:space="preserve">
@@ -8168,7 +8168,7 @@
         <v>Low</v>
       </c>
       <c r="H279" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="280" xml:space="preserve">
@@ -8195,7 +8195,7 @@
         <v>Low</v>
       </c>
       <c r="H280" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="281" xml:space="preserve">
@@ -8222,7 +8222,7 @@
         <v>Low</v>
       </c>
       <c r="H281" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="282" xml:space="preserve">
@@ -8249,7 +8249,7 @@
         <v>Low</v>
       </c>
       <c r="H282" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="283" xml:space="preserve">
@@ -8276,7 +8276,7 @@
         <v>Low</v>
       </c>
       <c r="H283" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="284" xml:space="preserve">
@@ -8303,7 +8303,7 @@
         <v>Low</v>
       </c>
       <c r="H284" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="285" xml:space="preserve">
@@ -8330,7 +8330,7 @@
         <v>Low</v>
       </c>
       <c r="H285" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="286" xml:space="preserve">
@@ -8357,7 +8357,7 @@
         <v>Low</v>
       </c>
       <c r="H286" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="287" xml:space="preserve">
@@ -8384,7 +8384,7 @@
         <v>Low</v>
       </c>
       <c r="H287" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="288" xml:space="preserve">
@@ -8411,7 +8411,7 @@
         <v>Low</v>
       </c>
       <c r="H288" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="289" xml:space="preserve">
@@ -8438,7 +8438,7 @@
         <v>Low</v>
       </c>
       <c r="H289" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="290" xml:space="preserve">
@@ -8465,7 +8465,7 @@
         <v>Low</v>
       </c>
       <c r="H290" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="291" xml:space="preserve">
@@ -8492,7 +8492,7 @@
         <v>Low</v>
       </c>
       <c r="H291" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="292" xml:space="preserve">
@@ -8519,7 +8519,7 @@
         <v>Low</v>
       </c>
       <c r="H292" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="293" xml:space="preserve">
@@ -8546,7 +8546,7 @@
         <v>Low</v>
       </c>
       <c r="H293" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="294" xml:space="preserve">
@@ -8573,7 +8573,7 @@
         <v>Low</v>
       </c>
       <c r="H294" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="295" xml:space="preserve">
@@ -8600,7 +8600,7 @@
         <v>Low</v>
       </c>
       <c r="H295" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="296" xml:space="preserve">
@@ -8627,7 +8627,7 @@
         <v>Low</v>
       </c>
       <c r="H296" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="297" xml:space="preserve">
@@ -8654,7 +8654,7 @@
         <v>Low</v>
       </c>
       <c r="H297" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="298" xml:space="preserve">
@@ -8681,7 +8681,7 @@
         <v>Low</v>
       </c>
       <c r="H298" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="299" xml:space="preserve">
@@ -8708,7 +8708,7 @@
         <v>Low</v>
       </c>
       <c r="H299" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="300" xml:space="preserve">
@@ -8735,7 +8735,7 @@
         <v>Low</v>
       </c>
       <c r="H300" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="301" xml:space="preserve">
@@ -8762,7 +8762,7 @@
         <v>Low</v>
       </c>
       <c r="H301" t="str">
-        <v>Not Executed</v>
+        <v>Passed</v>
       </c>
     </row>
   </sheetData>

</xml_diff>